<commit_message>
Replace legacy app entirely with source selector interface
</commit_message>
<xml_diff>
--- a/data/food.xlsx
+++ b/data/food.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="43">
   <si>
     <t>Restaurant</t>
   </si>
@@ -140,45 +140,6 @@
   </si>
   <si>
     <t>10:30~20:00</t>
-  </si>
-  <si>
-    <t>紅吱吱牛排館光復店</t>
-  </si>
-  <si>
-    <t>美式料理, 牛排</t>
-  </si>
-  <si>
-    <t>11:30~21:00</t>
-  </si>
-  <si>
-    <t>奉餡・汁心餃子：新竹清大店</t>
-  </si>
-  <si>
-    <t>中式料理, 麵食, 水餃, 煎餃</t>
-  </si>
-  <si>
-    <t>11:00~21:00</t>
-  </si>
-  <si>
-    <t>立晉豆花</t>
-  </si>
-  <si>
-    <t>豆花, 甜點, 冰</t>
-  </si>
-  <si>
-    <t>12:00~00:00</t>
-  </si>
-  <si>
-    <t>每週一暫停營業</t>
-  </si>
-  <si>
-    <t>六扇門時尚湯鍋 新竹建功店</t>
-  </si>
-  <si>
-    <t>火鍋</t>
-  </si>
-  <si>
-    <t>11:00~00:00</t>
   </si>
 </sst>
 </file>
@@ -930,34 +891,16 @@
       <c r="Z11" s="3"/>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D12" s="1">
-        <v>2.5</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
       <c r="H12" s="3"/>
-      <c r="I12" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>45</v>
-      </c>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
       <c r="K12" s="3"/>
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
@@ -976,28 +919,16 @@
       <c r="Z12" s="3"/>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D13" s="1">
-        <v>2.0</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
-      <c r="J13" s="1" t="s">
-        <v>48</v>
-      </c>
+      <c r="J13" s="3"/>
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
@@ -1016,35 +947,17 @@
       <c r="Z13" s="3"/>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D14" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
       <c r="G14" s="3"/>
-      <c r="H14" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="H14" s="3"/>
       <c r="I14" s="3"/>
-      <c r="J14" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>52</v>
-      </c>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
@@ -1062,34 +975,16 @@
       <c r="Z14" s="3"/>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="D15" s="1">
-        <v>2.5</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
       <c r="I15" s="3"/>
-      <c r="J15" s="1" t="s">
-        <v>55</v>
-      </c>
+      <c r="J15" s="3"/>
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
@@ -28100,6 +27995,9 @@
       <c r="Z979" s="3"/>
     </row>
     <row r="980">
+      <c r="A980" s="3"/>
+      <c r="B980" s="3"/>
+      <c r="C980" s="3"/>
       <c r="D980" s="3"/>
       <c r="E980" s="3"/>
       <c r="F980" s="3"/>
@@ -28125,6 +28023,9 @@
       <c r="Z980" s="3"/>
     </row>
     <row r="981">
+      <c r="A981" s="3"/>
+      <c r="B981" s="3"/>
+      <c r="C981" s="3"/>
       <c r="D981" s="3"/>
       <c r="E981" s="3"/>
       <c r="F981" s="3"/>
@@ -28150,6 +28051,9 @@
       <c r="Z981" s="3"/>
     </row>
     <row r="982">
+      <c r="A982" s="3"/>
+      <c r="B982" s="3"/>
+      <c r="C982" s="3"/>
       <c r="D982" s="3"/>
       <c r="E982" s="3"/>
       <c r="F982" s="3"/>
@@ -28175,6 +28079,9 @@
       <c r="Z982" s="3"/>
     </row>
     <row r="983">
+      <c r="A983" s="3"/>
+      <c r="B983" s="3"/>
+      <c r="C983" s="3"/>
       <c r="D983" s="3"/>
       <c r="E983" s="3"/>
       <c r="F983" s="3"/>
@@ -28200,6 +28107,9 @@
       <c r="Z983" s="3"/>
     </row>
     <row r="984">
+      <c r="A984" s="3"/>
+      <c r="B984" s="3"/>
+      <c r="C984" s="3"/>
       <c r="D984" s="3"/>
       <c r="E984" s="3"/>
       <c r="F984" s="3"/>
@@ -28225,6 +28135,9 @@
       <c r="Z984" s="3"/>
     </row>
     <row r="985">
+      <c r="A985" s="3"/>
+      <c r="B985" s="3"/>
+      <c r="C985" s="3"/>
       <c r="D985" s="3"/>
       <c r="E985" s="3"/>
       <c r="F985" s="3"/>
@@ -28250,6 +28163,9 @@
       <c r="Z985" s="3"/>
     </row>
     <row r="986">
+      <c r="A986" s="3"/>
+      <c r="B986" s="3"/>
+      <c r="C986" s="3"/>
       <c r="D986" s="3"/>
       <c r="E986" s="3"/>
       <c r="F986" s="3"/>
@@ -28449,13 +28365,188 @@
       <c r="Y993" s="3"/>
       <c r="Z993" s="3"/>
     </row>
+    <row r="994">
+      <c r="D994" s="3"/>
+      <c r="E994" s="3"/>
+      <c r="F994" s="3"/>
+      <c r="G994" s="3"/>
+      <c r="H994" s="3"/>
+      <c r="I994" s="3"/>
+      <c r="J994" s="3"/>
+      <c r="K994" s="3"/>
+      <c r="L994" s="3"/>
+      <c r="M994" s="3"/>
+      <c r="N994" s="3"/>
+      <c r="O994" s="3"/>
+      <c r="P994" s="3"/>
+      <c r="Q994" s="3"/>
+      <c r="R994" s="3"/>
+      <c r="S994" s="3"/>
+      <c r="T994" s="3"/>
+      <c r="U994" s="3"/>
+      <c r="V994" s="3"/>
+      <c r="W994" s="3"/>
+      <c r="X994" s="3"/>
+      <c r="Y994" s="3"/>
+      <c r="Z994" s="3"/>
+    </row>
+    <row r="995">
+      <c r="D995" s="3"/>
+      <c r="E995" s="3"/>
+      <c r="F995" s="3"/>
+      <c r="G995" s="3"/>
+      <c r="H995" s="3"/>
+      <c r="I995" s="3"/>
+      <c r="J995" s="3"/>
+      <c r="K995" s="3"/>
+      <c r="L995" s="3"/>
+      <c r="M995" s="3"/>
+      <c r="N995" s="3"/>
+      <c r="O995" s="3"/>
+      <c r="P995" s="3"/>
+      <c r="Q995" s="3"/>
+      <c r="R995" s="3"/>
+      <c r="S995" s="3"/>
+      <c r="T995" s="3"/>
+      <c r="U995" s="3"/>
+      <c r="V995" s="3"/>
+      <c r="W995" s="3"/>
+      <c r="X995" s="3"/>
+      <c r="Y995" s="3"/>
+      <c r="Z995" s="3"/>
+    </row>
+    <row r="996">
+      <c r="D996" s="3"/>
+      <c r="E996" s="3"/>
+      <c r="F996" s="3"/>
+      <c r="G996" s="3"/>
+      <c r="H996" s="3"/>
+      <c r="I996" s="3"/>
+      <c r="J996" s="3"/>
+      <c r="K996" s="3"/>
+      <c r="L996" s="3"/>
+      <c r="M996" s="3"/>
+      <c r="N996" s="3"/>
+      <c r="O996" s="3"/>
+      <c r="P996" s="3"/>
+      <c r="Q996" s="3"/>
+      <c r="R996" s="3"/>
+      <c r="S996" s="3"/>
+      <c r="T996" s="3"/>
+      <c r="U996" s="3"/>
+      <c r="V996" s="3"/>
+      <c r="W996" s="3"/>
+      <c r="X996" s="3"/>
+      <c r="Y996" s="3"/>
+      <c r="Z996" s="3"/>
+    </row>
+    <row r="997">
+      <c r="D997" s="3"/>
+      <c r="E997" s="3"/>
+      <c r="F997" s="3"/>
+      <c r="G997" s="3"/>
+      <c r="H997" s="3"/>
+      <c r="I997" s="3"/>
+      <c r="J997" s="3"/>
+      <c r="K997" s="3"/>
+      <c r="L997" s="3"/>
+      <c r="M997" s="3"/>
+      <c r="N997" s="3"/>
+      <c r="O997" s="3"/>
+      <c r="P997" s="3"/>
+      <c r="Q997" s="3"/>
+      <c r="R997" s="3"/>
+      <c r="S997" s="3"/>
+      <c r="T997" s="3"/>
+      <c r="U997" s="3"/>
+      <c r="V997" s="3"/>
+      <c r="W997" s="3"/>
+      <c r="X997" s="3"/>
+      <c r="Y997" s="3"/>
+      <c r="Z997" s="3"/>
+    </row>
+    <row r="998">
+      <c r="D998" s="3"/>
+      <c r="E998" s="3"/>
+      <c r="F998" s="3"/>
+      <c r="G998" s="3"/>
+      <c r="H998" s="3"/>
+      <c r="I998" s="3"/>
+      <c r="J998" s="3"/>
+      <c r="K998" s="3"/>
+      <c r="L998" s="3"/>
+      <c r="M998" s="3"/>
+      <c r="N998" s="3"/>
+      <c r="O998" s="3"/>
+      <c r="P998" s="3"/>
+      <c r="Q998" s="3"/>
+      <c r="R998" s="3"/>
+      <c r="S998" s="3"/>
+      <c r="T998" s="3"/>
+      <c r="U998" s="3"/>
+      <c r="V998" s="3"/>
+      <c r="W998" s="3"/>
+      <c r="X998" s="3"/>
+      <c r="Y998" s="3"/>
+      <c r="Z998" s="3"/>
+    </row>
+    <row r="999">
+      <c r="D999" s="3"/>
+      <c r="E999" s="3"/>
+      <c r="F999" s="3"/>
+      <c r="G999" s="3"/>
+      <c r="H999" s="3"/>
+      <c r="I999" s="3"/>
+      <c r="J999" s="3"/>
+      <c r="K999" s="3"/>
+      <c r="L999" s="3"/>
+      <c r="M999" s="3"/>
+      <c r="N999" s="3"/>
+      <c r="O999" s="3"/>
+      <c r="P999" s="3"/>
+      <c r="Q999" s="3"/>
+      <c r="R999" s="3"/>
+      <c r="S999" s="3"/>
+      <c r="T999" s="3"/>
+      <c r="U999" s="3"/>
+      <c r="V999" s="3"/>
+      <c r="W999" s="3"/>
+      <c r="X999" s="3"/>
+      <c r="Y999" s="3"/>
+      <c r="Z999" s="3"/>
+    </row>
+    <row r="1000">
+      <c r="D1000" s="3"/>
+      <c r="E1000" s="3"/>
+      <c r="F1000" s="3"/>
+      <c r="G1000" s="3"/>
+      <c r="H1000" s="3"/>
+      <c r="I1000" s="3"/>
+      <c r="J1000" s="3"/>
+      <c r="K1000" s="3"/>
+      <c r="L1000" s="3"/>
+      <c r="M1000" s="3"/>
+      <c r="N1000" s="3"/>
+      <c r="O1000" s="3"/>
+      <c r="P1000" s="3"/>
+      <c r="Q1000" s="3"/>
+      <c r="R1000" s="3"/>
+      <c r="S1000" s="3"/>
+      <c r="T1000" s="3"/>
+      <c r="U1000" s="3"/>
+      <c r="V1000" s="3"/>
+      <c r="W1000" s="3"/>
+      <c r="X1000" s="3"/>
+      <c r="Y1000" s="3"/>
+      <c r="Z1000" s="3"/>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B15">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C11">
+      <formula1>"早餐,早午餐,中式料理,美式料理,炸物,速食,義式料理,義大利麵,焗烤,超商,異國美食,便當,麵食,丼飯,咖哩,飲料,水果,牛奶"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B11">
       <formula1>"小吃部,風雲樓,水木,清夜"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C15">
-      <formula1>"早餐,早午餐,中式料理,美式料理,炸物,速食,義式料理,義大利麵,焗烤,超商,異國美食,便當,麵食,丼飯,咖哩,飲料,水果,牛奶,牛排,水餃,煎餃,豆花,甜點,冰,火鍋"</formula1>
     </dataValidation>
   </dataValidations>
   <drawing r:id="rId1"/>

</xml_diff>